<commit_message>
fix(ui): improve AnalysisTab columns, pagination and mock excel
</commit_message>
<xml_diff>
--- a/Consolidado_Mock_10A.xlsx
+++ b/Consolidado_Mock_10A.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:AF8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,27 +431,66 @@
         <v/>
       </c>
       <c r="K1" t="str">
+        <v/>
+      </c>
+      <c r="L1" t="str">
+        <v/>
+      </c>
+      <c r="M1" t="str">
+        <v/>
+      </c>
+      <c r="N1" t="str">
         <v>MATEMATICAS</v>
       </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v/>
-      </c>
-      <c r="N1" t="str">
-        <v/>
-      </c>
       <c r="O1" t="str">
+        <v/>
+      </c>
+      <c r="P1" t="str">
+        <v/>
+      </c>
+      <c r="Q1" t="str">
+        <v/>
+      </c>
+      <c r="R1" t="str">
+        <v/>
+      </c>
+      <c r="S1" t="str">
+        <v/>
+      </c>
+      <c r="T1" t="str">
+        <v/>
+      </c>
+      <c r="U1" t="str">
+        <v/>
+      </c>
+      <c r="V1" t="str">
+        <v/>
+      </c>
+      <c r="W1" t="str">
         <v>HUMANIDADES</v>
       </c>
-      <c r="P1" t="str">
-        <v/>
-      </c>
-      <c r="Q1" t="str">
-        <v/>
-      </c>
-      <c r="R1" t="str">
+      <c r="X1" t="str">
+        <v/>
+      </c>
+      <c r="Y1" t="str">
+        <v/>
+      </c>
+      <c r="Z1" t="str">
+        <v/>
+      </c>
+      <c r="AA1" t="str">
+        <v/>
+      </c>
+      <c r="AB1" t="str">
+        <v/>
+      </c>
+      <c r="AC1" t="str">
+        <v/>
+      </c>
+      <c r="AD1" t="str">
+        <v/>
+      </c>
+      <c r="AE1" t="str">
         <v/>
       </c>
     </row>
@@ -487,28 +526,70 @@
         <v/>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v>DEF</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>ALGEBRA</v>
       </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v>GEOMETRIA</v>
       </c>
-      <c r="O2" t="str">
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v>DEF</v>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
         <v>LENGUAJE</v>
       </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
         <v>INGLES</v>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v>DEF</v>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -543,16 +624,16 @@
         <v>P2</v>
       </c>
       <c r="K3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L3" t="str">
         <v>P1</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>P2</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>P3</v>
-      </c>
-      <c r="N3" t="str">
-        <v>P1</v>
       </c>
       <c r="O3" t="str">
         <v>P1</v>
@@ -565,6 +646,48 @@
       </c>
       <c r="R3" t="str">
         <v>P1</v>
+      </c>
+      <c r="S3" t="str">
+        <v>P2</v>
+      </c>
+      <c r="T3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="U3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="V3" t="str">
+        <v>P2</v>
+      </c>
+      <c r="W3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="X3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>P2</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>P2</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>P2</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>P3</v>
       </c>
     </row>
     <row r="4">
@@ -580,8 +703,8 @@
       <c r="D4">
         <v>4</v>
       </c>
-      <c r="E4" t="str">
-        <v/>
+      <c r="E4">
+        <v>4.2</v>
       </c>
       <c r="F4">
         <v>3.8</v>
@@ -589,8 +712,8 @@
       <c r="G4">
         <v>4.2</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
+      <c r="H4">
+        <v>4</v>
       </c>
       <c r="I4">
         <v>4</v>
@@ -599,28 +722,70 @@
         <v>4.1</v>
       </c>
       <c r="K4">
+        <v>4.1</v>
+      </c>
+      <c r="L4">
+        <v>4.1</v>
+      </c>
+      <c r="M4">
+        <v>4.1</v>
+      </c>
+      <c r="N4">
+        <v>4.1</v>
+      </c>
+      <c r="O4">
         <v>4.5</v>
       </c>
-      <c r="L4">
+      <c r="P4">
         <v>4.8</v>
       </c>
-      <c r="M4" t="str">
-        <v/>
-      </c>
-      <c r="N4">
-        <v>4</v>
-      </c>
-      <c r="O4">
+      <c r="Q4">
+        <v>4.6</v>
+      </c>
+      <c r="R4">
+        <v>4</v>
+      </c>
+      <c r="S4">
         <v>3.5</v>
       </c>
-      <c r="P4">
+      <c r="T4">
         <v>3.8</v>
       </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4">
+      <c r="U4">
         <v>4.2</v>
+      </c>
+      <c r="V4">
+        <v>4.1</v>
+      </c>
+      <c r="W4">
+        <v>4.2</v>
+      </c>
+      <c r="X4">
+        <v>3.8</v>
+      </c>
+      <c r="Y4">
+        <v>4</v>
+      </c>
+      <c r="Z4">
+        <v>3.9</v>
+      </c>
+      <c r="AA4">
+        <v>4.2</v>
+      </c>
+      <c r="AB4">
+        <v>4.5</v>
+      </c>
+      <c r="AC4">
+        <v>4.3</v>
+      </c>
+      <c r="AD4">
+        <v>4</v>
+      </c>
+      <c r="AE4">
+        <v>4.2</v>
+      </c>
+      <c r="AF4">
+        <v>4.1</v>
       </c>
     </row>
     <row r="5">
@@ -636,8 +801,8 @@
       <c r="D5">
         <v>2.5</v>
       </c>
-      <c r="E5" t="str">
-        <v/>
+      <c r="E5">
+        <v>2.8</v>
       </c>
       <c r="F5">
         <v>2.8</v>
@@ -645,8 +810,8 @@
       <c r="G5">
         <v>3.1</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
+      <c r="H5">
+        <v>3</v>
       </c>
       <c r="I5">
         <v>2.5</v>
@@ -655,28 +820,70 @@
         <v>2</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>2.2</v>
       </c>
       <c r="L5">
+        <v>2.7</v>
+      </c>
+      <c r="M5">
+        <v>2.5</v>
+      </c>
+      <c r="N5">
+        <v>2.6</v>
+      </c>
+      <c r="O5">
+        <v>4</v>
+      </c>
+      <c r="P5">
         <v>3.8</v>
       </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5">
+      <c r="Q5">
+        <v>3.9</v>
+      </c>
+      <c r="R5">
         <v>3.5</v>
       </c>
-      <c r="O5">
-        <v>4</v>
-      </c>
-      <c r="P5">
+      <c r="S5">
+        <v>4</v>
+      </c>
+      <c r="T5">
+        <v>3.8</v>
+      </c>
+      <c r="U5">
+        <v>3.7</v>
+      </c>
+      <c r="V5">
+        <v>3.9</v>
+      </c>
+      <c r="W5">
+        <v>3.8</v>
+      </c>
+      <c r="X5">
         <v>4.2</v>
       </c>
-      <c r="Q5" t="str">
-        <v/>
-      </c>
-      <c r="R5">
+      <c r="Y5">
         <v>3.8</v>
+      </c>
+      <c r="Z5">
+        <v>4</v>
+      </c>
+      <c r="AA5">
+        <v>3.8</v>
+      </c>
+      <c r="AB5">
+        <v>4</v>
+      </c>
+      <c r="AC5">
+        <v>3.9</v>
+      </c>
+      <c r="AD5">
+        <v>4</v>
+      </c>
+      <c r="AE5">
+        <v>3.9</v>
+      </c>
+      <c r="AF5">
+        <v>3.9</v>
       </c>
     </row>
     <row r="6">
@@ -692,8 +899,8 @@
       <c r="D6">
         <v>3.8</v>
       </c>
-      <c r="E6" t="str">
-        <v/>
+      <c r="E6">
+        <v>3.6</v>
       </c>
       <c r="F6">
         <v>3.9</v>
@@ -701,8 +908,8 @@
       <c r="G6">
         <v>4</v>
       </c>
-      <c r="H6" t="str">
-        <v/>
+      <c r="H6">
+        <v>3.9</v>
       </c>
       <c r="I6">
         <v>3.5</v>
@@ -711,28 +918,70 @@
         <v>3.6</v>
       </c>
       <c r="K6">
+        <v>3.5</v>
+      </c>
+      <c r="L6">
+        <v>3.6</v>
+      </c>
+      <c r="M6">
+        <v>3.8</v>
+      </c>
+      <c r="N6">
+        <v>3.6</v>
+      </c>
+      <c r="O6">
         <v>1.5</v>
       </c>
-      <c r="L6">
+      <c r="P6">
         <v>2</v>
       </c>
-      <c r="M6" t="str">
-        <v/>
-      </c>
-      <c r="N6">
+      <c r="Q6">
+        <v>1.8</v>
+      </c>
+      <c r="R6">
         <v>2</v>
       </c>
-      <c r="O6">
+      <c r="S6">
         <v>3</v>
       </c>
-      <c r="P6">
+      <c r="T6">
+        <v>2.5</v>
+      </c>
+      <c r="U6">
+        <v>1.7</v>
+      </c>
+      <c r="V6">
+        <v>2.5</v>
+      </c>
+      <c r="W6">
+        <v>2.1</v>
+      </c>
+      <c r="X6">
         <v>3.2</v>
       </c>
-      <c r="Q6" t="str">
-        <v/>
-      </c>
-      <c r="R6">
+      <c r="Y6">
         <v>3</v>
+      </c>
+      <c r="Z6">
+        <v>3.1</v>
+      </c>
+      <c r="AA6">
+        <v>3</v>
+      </c>
+      <c r="AB6">
+        <v>3.5</v>
+      </c>
+      <c r="AC6">
+        <v>3.2</v>
+      </c>
+      <c r="AD6">
+        <v>3.1</v>
+      </c>
+      <c r="AE6">
+        <v>3.2</v>
+      </c>
+      <c r="AF6">
+        <v>3.1</v>
       </c>
     </row>
     <row r="7">
@@ -748,8 +997,8 @@
       <c r="D7">
         <v>4.2</v>
       </c>
-      <c r="E7" t="str">
-        <v/>
+      <c r="E7">
+        <v>4.1</v>
       </c>
       <c r="F7">
         <v>3.5</v>
@@ -757,8 +1006,8 @@
       <c r="G7">
         <v>3</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
+      <c r="H7">
+        <v>3.2</v>
       </c>
       <c r="I7">
         <v>4.8</v>
@@ -767,28 +1016,70 @@
         <v>4.5</v>
       </c>
       <c r="K7">
+        <v>4.6</v>
+      </c>
+      <c r="L7">
+        <v>4.1</v>
+      </c>
+      <c r="M7">
+        <v>3.9</v>
+      </c>
+      <c r="N7">
+        <v>3.9</v>
+      </c>
+      <c r="O7">
         <v>3.2</v>
       </c>
-      <c r="L7">
+      <c r="P7">
         <v>3.5</v>
       </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-      <c r="N7">
+      <c r="Q7">
+        <v>3.3</v>
+      </c>
+      <c r="R7">
         <v>3.8</v>
       </c>
-      <c r="O7">
+      <c r="S7">
         <v>4.5</v>
       </c>
-      <c r="P7">
+      <c r="T7">
+        <v>4.1</v>
+      </c>
+      <c r="U7">
+        <v>3.5</v>
+      </c>
+      <c r="V7">
+        <v>4</v>
+      </c>
+      <c r="W7">
+        <v>3.7</v>
+      </c>
+      <c r="X7">
         <v>4.8</v>
       </c>
-      <c r="Q7" t="str">
-        <v/>
-      </c>
-      <c r="R7">
+      <c r="Y7">
         <v>4.6</v>
+      </c>
+      <c r="Z7">
+        <v>4.7</v>
+      </c>
+      <c r="AA7">
+        <v>4.2</v>
+      </c>
+      <c r="AB7">
+        <v>4</v>
+      </c>
+      <c r="AC7">
+        <v>4.1</v>
+      </c>
+      <c r="AD7">
+        <v>4.5</v>
+      </c>
+      <c r="AE7">
+        <v>4.3</v>
+      </c>
+      <c r="AF7">
+        <v>4.4</v>
       </c>
     </row>
     <row r="8">
@@ -822,34 +1113,76 @@
       <c r="J8">
         <v>2.8</v>
       </c>
-      <c r="K8">
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8">
+        <v>2.9</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8">
         <v>3.5</v>
       </c>
-      <c r="L8" t="str">
-        <v/>
-      </c>
-      <c r="M8" t="str">
-        <v/>
-      </c>
-      <c r="N8">
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8">
         <v>3</v>
       </c>
-      <c r="O8">
-        <v>4</v>
-      </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-      <c r="Q8" t="str">
-        <v/>
-      </c>
-      <c r="R8">
+      <c r="S8">
+        <v>4</v>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8">
+        <v>3.2</v>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8">
         <v>3.5</v>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>